<commit_message>
Excel previews in Segoe UI; budget label width and palette-correct critical shade
Previews re-rendered with the real Segoe UI. The budget summary's adjustment column is
wider so its labels don't clip, and the scoping workbook flags critical risk in Indigo
Lightest #D9C9F7 from the palette. serve.py can serve another folder (for the Frame
review package).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/assets/downloads/SmartCommunications_Budget_Planning_Template.xlsx
+++ b/site/assets/downloads/SmartCommunications_Budget_Planning_Template.xlsx
@@ -670,7 +670,7 @@
       <row>0</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="19135725" cy="609600"/>
+    <ext cx="19411950" cy="609600"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -1541,7 +1541,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>

</xml_diff>